<commit_message>
Refatoração completa da V3: motor centralizado e limpeza de redundâncias
</commit_message>
<xml_diff>
--- a/data/DadosSedimentation.xlsx
+++ b/data/DadosSedimentation.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Izaq\Projects\optigen-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9C2A18-2F22-4BBA-B628-FCC6B2FF1D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598A4703-94D4-44A2-A468-0C8B92535462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7C89A78E-0117-400B-BF16-4A00B9D07968}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7C89A78E-0117-400B-BF16-4A00B9D07968}"/>
   </bookViews>
   <sheets>
     <sheet name="fluids_meta" sheetId="2" r:id="rId1"/>
     <sheet name="measurements" sheetId="1" r:id="rId2"/>
-    <sheet name="Planilha1" sheetId="3" r:id="rId3"/>
+    <sheet name="info" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>ROA</t>
   </si>
@@ -92,6 +92,12 @@
   </si>
   <si>
     <t>dp_medio D50 (μm)</t>
+  </si>
+  <si>
+    <t>altura(cm)</t>
+  </si>
+  <si>
+    <t>tempo (dia)</t>
   </si>
 </sst>
 </file>
@@ -34358,7 +34364,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72CB93C3-27B4-46B4-8B18-76E97D9C21F4}">
-  <dimension ref="B3:J9"/>
+  <dimension ref="B3:M9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="4.5546875" bestFit="1" customWidth="1"/>
@@ -34366,9 +34372,11 @@
     <col min="6" max="6" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
@@ -34396,8 +34404,14 @@
       <c r="J3" s="12" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="L3" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B4" s="11">
         <v>5</v>
       </c>
@@ -34426,7 +34440,7 @@
         <v>0.39700000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B5" s="11">
         <v>6</v>
       </c>
@@ -34455,7 +34469,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B6" s="11">
         <v>7</v>
       </c>
@@ -34484,7 +34498,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B7" s="11">
         <v>8</v>
       </c>
@@ -34513,7 +34527,7 @@
         <v>0.20100000000000001</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B8" s="11">
         <v>9</v>
       </c>
@@ -34543,7 +34557,7 @@
         <v>0.47199999999999998</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B9" s="11">
         <v>10</v>
       </c>

</xml_diff>